<commit_message>
Added test scripts in homePageTest
</commit_message>
<xml_diff>
--- a/src/test/resources/test-data/testData.xlsx
+++ b/src/test/resources/test-data/testData.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ashok\IdeaProjects\CucumberDemoProject\src\test\resources\test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D84F491F-16A0-4B9F-8894-1CA662998419}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F884E42-350F-49B5-AD58-48F23DBF4B7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="LoginPage" sheetId="1" r:id="rId1"/>
+    <sheet name="HomePage" sheetId="2" r:id="rId1"/>
+    <sheet name="LoginPage" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>username</t>
   </si>
@@ -37,13 +38,52 @@
   </si>
   <si>
     <t>EdApYze</t>
+  </si>
+  <si>
+    <t>MenuList</t>
+  </si>
+  <si>
+    <t>Manager</t>
+  </si>
+  <si>
+    <t>New Customer</t>
+  </si>
+  <si>
+    <t>Edit Customer</t>
+  </si>
+  <si>
+    <t>Delete Customer</t>
+  </si>
+  <si>
+    <t>New Account</t>
+  </si>
+  <si>
+    <t>Edit Account</t>
+  </si>
+  <si>
+    <t>Delete Account</t>
+  </si>
+  <si>
+    <t>Mini Statement</t>
+  </si>
+  <si>
+    <t>Log out</t>
+  </si>
+  <si>
+    <t>Heading Loop</t>
+  </si>
+  <si>
+    <t>Welcome to Manager's Page of GTPL Bank</t>
+  </si>
+  <si>
+    <t>Customised Statement</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -57,6 +97,14 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -79,9 +127,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -361,6 +410,90 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82B9C20C-3B37-49ED-90FA-323221C79A75}">
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="18.59765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34.3984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.9296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.19921875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.06640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.59765625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>

</xml_diff>